<commit_message>
Enriquecer base de datos con contenido real verificado de WordPress
70 temas verificados via API REST de WordPress. Keywords actualizadas con contenido real extraído de cada tema. Nueva columna: Tiene Video y Contenido Real Verificado.
</commit_message>
<xml_diff>
--- a/quimica_ucv_base_datos.xlsx
+++ b/quimica_ucv_base_datos.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -518,6 +518,16 @@
           <t>Descripción para IA</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Tiene Video</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Contenido Real Verificado</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -586,12 +596,22 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>materia, energía, estados de la materia, propiedades, clasificación, sustancias puras, mezclas</t>
+          <t>materia, energía, estados de la materia, propiedades, clasificación, sustancias puras, mezclas, conceptos básicos química, materia energía, propiedades, clasificación, estados materia, sustancias puras mezclas, h5p interactivo</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Tema sobre materia y energía: clasificación de la materia, estados, propiedades físicas y químicas, tipos de energía</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>conceptos básicos química, materia energía, propiedades, clasificación, estados materia, sustancias puras mezclas, h5p interactivo</t>
         </is>
       </c>
     </row>
@@ -662,12 +682,22 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>óxidos, óxidos básicos, óxidos ácidos, anhídridos, compuestos oxigenados, nomenclatura</t>
+          <t>óxidos, óxidos básicos, óxidos ácidos, anhídridos, compuestos oxigenados, nomenclatura, formular nombrar compuestos oxigenados, óxidos básicos ácidos anhídridos, nomenclatura IUPAC stock tradicional números oxidación</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Compuestos oxigenados: óxidos básicos y ácidos, nomenclatura IUPAC, stock y tradicional</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>formular nombrar compuestos oxigenados, óxidos básicos ácidos anhídridos, nomenclatura IUPAC stock tradicional números oxidación</t>
         </is>
       </c>
     </row>
@@ -702,12 +732,22 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>hidruros, compuestos hidrogenados, hidrógeno, hidruros metálicos, hidruros no metálicos</t>
+          <t>hidruros, compuestos hidrogenados, hidrógeno, hidruros metálicos, hidruros no metálicos, formular nombrar compuestos hidrogenados, hidruros metálicos, hidrógeno combinado otros elementos</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Compuestos hidrogenados: hidruros metálicos y no metálicos, nomenclatura y formulación</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>formular nombrar compuestos hidrogenados, hidruros metálicos, hidrógeno combinado otros elementos</t>
         </is>
       </c>
     </row>
@@ -742,12 +782,22 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>sales binarias, haluros, sulfuros, compuestos binarios, metal + no metal</t>
+          <t>sales binarias, haluros, sulfuros, compuestos binarios, metal + no metal, formular nombrar sales binarias, metal + no metal, sin oxígeno, números oxidación intercambio</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Sales binarias: combinación de metal con no metal, haluros, sulfuros, nomenclatura</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>formular nombrar sales binarias, metal + no metal, sin oxígeno, números oxidación intercambio</t>
         </is>
       </c>
     </row>
@@ -782,12 +832,22 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>hidróxidos, bases, grupo hidroxilo, OH, compuestos básicos, nomenclatura</t>
+          <t>hidróxidos, bases, grupo hidroxilo, OH, compuestos básicos, nomenclatura, formular nombrar hidróxidos, metal + grupo hidroxilo OH, números oxidación intercambio valencias</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Hidróxidos o bases: formación, nomenclatura, grupo OH, propiedades básicas</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>formular nombrar hidróxidos, metal + grupo hidroxilo OH, números oxidación intercambio valencias</t>
         </is>
       </c>
     </row>
@@ -822,12 +882,22 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>ácidos oxácidos, oxoácidos, hidrógeno + no metal + oxígeno, nomenclatura</t>
+          <t>ácidos oxácidos, oxoácidos, hidrógeno + no metal + oxígeno, nomenclatura, formular nombrar ácidos oxácidos, hidrógeno oxígeno no metal, números oxidación reglas formulación</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Ácidos oxácidos: formación a partir de anhídridos + agua, nomenclatura IUPAC y tradicional</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>formular nombrar ácidos oxácidos, hidrógeno oxígeno no metal, números oxidación reglas formulación</t>
         </is>
       </c>
     </row>
@@ -862,12 +932,22 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>sales neutras, oxisales, neutralización, metal + radical ácido</t>
+          <t>sales neutras, oxisales, neutralización, metal + radical ácido, formular nombrar sales neutras oxisales, neutralización total ácido base, catión anión</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Sales neutras: formación por neutralización total, nomenclatura de oxisales</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>formular nombrar sales neutras oxisales, neutralización total ácido base, catión anión</t>
         </is>
       </c>
     </row>
@@ -902,12 +982,22 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>sales ácidas, hidrógeno, neutralización parcial, bisales</t>
+          <t>sales ácidas, hidrógeno, neutralización parcial, bisales, sales ácidas neutralización parcial, hidrógeno restante bisales</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Sales ácidas: neutralización parcial de ácidos polipróticos, nomenclatura con hidrógeno</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>sales ácidas neutralización parcial, hidrógeno restante bisales</t>
         </is>
       </c>
     </row>
@@ -942,12 +1032,22 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>sales básicas, hidroxisales, grupo OH, neutralización parcial de bases</t>
+          <t>sales básicas, hidroxisales, grupo OH, neutralización parcial de bases, sales básicas hidroxisales, neutralización parcial bases, grupo OH restante</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Sales básicas: formación por neutralización parcial de bases, hidroxisales</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>sales básicas hidroxisales, neutralización parcial bases, grupo OH restante</t>
         </is>
       </c>
     </row>
@@ -1018,12 +1118,22 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>peso molecular, masa molecular relativa, uma, masa atómica, tabla periódica, cálculo</t>
+          <t>peso molecular, masa molecular relativa, uma, masa atómica, tabla periódica, cálculo, cálculo peso molecular usando tabla periódica, suma masas atómicas, uma, dalton</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Cálculo del peso molecular: sumar masas atómicas de cada elemento × cantidad de átomos</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>cálculo peso molecular usando tabla periódica, suma masas atómicas, uma, dalton</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1204,22 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>moles, átomos, gramos, Avogadro, 6.022×10²³, conversiones mol-átomo-gramo</t>
+          <t>moles, átomos, gramos, Avogadro, 6.022×10²³, conversiones mol-átomo-gramo, conversiones moles átomos gramos, número Avogadro 6.022x10^23</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Conversiones entre moles, átomos y gramos usando el número de Avogadro</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>conversiones moles átomos gramos, número Avogadro 6.022x10^23</t>
         </is>
       </c>
     </row>
@@ -1134,12 +1254,22 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>moles a gramos, gramos a moles, masa molar, conversión, peso molecular</t>
+          <t>moles a gramos, gramos a moles, masa molar, conversión, peso molecular, cómo está formada materia átomos, iones, unidades más pequeñas elementos, ganar perder electrones</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Conversión entre moles y gramos usando la masa molar como factor de conversión</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>cómo está formada materia átomos, iones, unidades más pequeñas elementos, ganar perder electrones</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1344,22 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>átomos a gramos, gramos a átomos, conversión directa, Avogadro, masa molar</t>
+          <t>átomos a gramos, gramos a átomos, conversión directa, Avogadro, masa molar, conversión directa átomos gramos, combinar Avogadro masa molar</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Conversión directa entre átomos y gramos combinando Avogadro y masa molar</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>conversión directa átomos gramos, combinar Avogadro masa molar</t>
         </is>
       </c>
     </row>
@@ -1254,12 +1394,22 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>moléculas, moles de moléculas, número de moléculas, Avogadro, conversión</t>
+          <t>moléculas, moles de moléculas, número de moléculas, Avogadro, conversión, concepto molécula, conversiones moles número moléculas, Avogadro</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Concepto de molécula y conversiones entre moles y número de moléculas</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>concepto molécula, conversiones moles número moléculas, Avogadro</t>
         </is>
       </c>
     </row>
@@ -1330,12 +1480,22 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>composición centesimal, porcentaje en masa, porcentaje de cada elemento, fórmula</t>
+          <t>composición centesimal, porcentaje en masa, porcentaje de cada elemento, fórmula, calcular composición centesimal porcentual paso a paso, porcentajes ejercicios</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Cálculo del porcentaje en masa de cada elemento en un compuesto químico</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>calcular composición centesimal porcentual paso a paso, porcentajes ejercicios</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1566,22 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>fórmula mínima, fórmula empírica, proporción mínima, moles, simplificar</t>
+          <t>fórmula mínima, fórmula empírica, proporción mínima, moles, simplificar, fórmula mínima molecular gases densidad volumen molar</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
           <t>Determinación de la fórmula mínima o empírica a partir de datos de composición</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>fórmula mínima molecular gases densidad volumen molar</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1616,22 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>fórmula molecular, fórmula real, múltiplo, fórmula mínima, peso molecular</t>
+          <t>fórmula molecular, fórmula real, múltiplo, fórmula mínima, peso molecular, fórmula mínima empírica, proporción mínima moles simplificar datos composición</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
           <t>Determinación de fórmula molecular: múltiplo entero de la fórmula mínima</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>fórmula mínima empírica, proporción mínima moles simplificar datos composición</t>
         </is>
       </c>
     </row>
@@ -1522,12 +1702,22 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>estequiometría, introducción, ecuaciones químicas, balanceo, coeficientes, relaciones molares</t>
+          <t>estequiometría, introducción, ecuaciones químicas, balanceo, coeficientes, relaciones molares, video estequiometría, balanceo ecuaciones químicas, relaciones molares, coeficientes</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
           <t>Introducción a la estequiometría: balanceo de ecuaciones y relaciones molares</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>video estequiometría, balanceo ecuaciones químicas, relaciones molares, coeficientes</t>
         </is>
       </c>
     </row>
@@ -1562,12 +1752,22 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>reactivo limitante, reactivo en exceso, rendimiento teórico, cantidad de producto</t>
+          <t>reactivo limitante, reactivo en exceso, rendimiento teórico, cantidad de producto, identificar reactivo limitante exceso, cálculo rendimiento teórico, cantidad producto</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
           <t>Identificación del reactivo limitante y en exceso, cálculo de rendimiento teórico</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>identificar reactivo limitante exceso, cálculo rendimiento teórico, cantidad producto</t>
         </is>
       </c>
     </row>
@@ -1642,12 +1842,22 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>rendimiento porcentual, rendimiento real, rendimiento teórico, porcentaje, eficiencia</t>
+          <t>rendimiento porcentual, rendimiento real, rendimiento teórico, porcentaje, eficiencia, rendimiento porcentual real teórico eficiencia reacción</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
           <t>Cálculo de rendimiento porcentual: relación entre rendimiento real y teórico</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>rendimiento porcentual real teórico eficiencia reacción</t>
         </is>
       </c>
     </row>
@@ -1682,12 +1892,22 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>estequiometría, soluciones, molaridad, volumen, concentración, reacciones en solución</t>
+          <t>estequiometría, soluciones, molaridad, volumen, concentración, reacciones en solución, estequiometría soluciones molaridad volumen reacciones en solución</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
           <t>Estequiometría aplicada a reacciones en solución usando molaridad y volumen</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>estequiometría soluciones molaridad volumen reacciones en solución</t>
         </is>
       </c>
     </row>
@@ -1722,12 +1942,22 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>estequiometría, fórmula mínima, fórmula empírica, cálculos combinados</t>
+          <t>estequiometría, fórmula mínima, fórmula empírica, cálculos combinados, fórmula mínima empírica, proporción mínima moles simplificar datos composición</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
           <t>Problemas que combinan estequiometría con determinación de fórmula mínima</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>fórmula mínima empírica, proporción mínima moles simplificar datos composición</t>
         </is>
       </c>
     </row>
@@ -1798,12 +2028,22 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>radio atómico, radio iónico, energía de ionización, tendencias periódicas, tamaño</t>
+          <t>radio atómico, radio iónico, energía de ionización, tendencias periódicas, tamaño, video sobre radio atómico radio iónico energía ionización tendencias periódicas</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
           <t>Propiedades periódicas: radio atómico, radio iónico y energía de ionización, tendencias en la tabla</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>video sobre radio atómico radio iónico energía ionización tendencias periódicas</t>
         </is>
       </c>
     </row>
@@ -1878,12 +2118,22 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>afinidad electrónica, electronegatividad, Pauling, tendencias, atracción de electrones</t>
+          <t>afinidad electrónica, electronegatividad, Pauling, tendencias, atracción de electrones, diferenciar afinidad electrónica electronegatividad, propiedades periódicas, cómo átomos atraen electrones, variación tabla periódica</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
           <t>Afinidad electrónica y electronegatividad: definiciones, escalas y tendencias periódicas</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>diferenciar afinidad electrónica electronegatividad, propiedades periódicas, cómo átomos atraen electrones, variación tabla periódica</t>
         </is>
       </c>
     </row>
@@ -1918,12 +2168,22 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>isótopos, isóbaros, isótonos, isoelectrónicos, número atómico, número másico, neutrones</t>
+          <t>isótopos, isóbaros, isótonos, isoelectrónicos, número atómico, número másico, neutrones, clasificación especies, isótopos mismo Z, isóbaros mismo A, isótonos mismo N, isoelectrónicos</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
           <t>Clasificación de especies: isótopos (mismo Z), isóbaros (mismo A), isótonos (mismo N), isoelectrónicos</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>clasificación especies, isótopos mismo Z, isóbaros mismo A, isótonos mismo N, isoelectrónicos</t>
         </is>
       </c>
     </row>
@@ -1958,12 +2218,22 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>abundancia isotópica, masa atómica promedio, isótopos, porcentaje natural</t>
+          <t>abundancia isotópica, masa atómica promedio, isótopos, porcentaje natural, cálculo masa atómica promedio, abundancia isotópica porcentaje natural</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
           <t>Cálculo de masa atómica promedio a partir de abundancia isotópica de cada isótopo</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>cálculo masa atómica promedio, abundancia isotópica porcentaje natural</t>
         </is>
       </c>
     </row>
@@ -2034,12 +2304,22 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>configuración electrónica, Aufbau, Hund, Pauli, subniveles, s p d f, diagrama de Moeller</t>
+          <t>configuración electrónica, Aufbau, Hund, Pauli, subniveles, s p d f, diagrama de Moeller, configuración electrónica, Aufbau, Hund, Pauli, subniveles s p d f, Moeller</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
           <t>Configuración electrónica: principio de Aufbau, regla de Hund, principio de exclusión de Pauli</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>configuración electrónica, Aufbau, Hund, Pauli, subniveles s p d f, Moeller</t>
         </is>
       </c>
     </row>
@@ -2074,12 +2354,22 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>excepciones, cromo, cobre, configuración anómala, estabilidad, semilleno, lleno</t>
+          <t>excepciones, cromo, cobre, configuración anómala, estabilidad, semilleno, lleno, configuración electrónica, Aufbau, Hund, Pauli, subniveles s p d f, Moeller</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
           <t>Excepciones en configuración electrónica: Cr, Cu y elementos de transición con subniveles d</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>configuración electrónica, Aufbau, Hund, Pauli, subniveles s p d f, Moeller</t>
         </is>
       </c>
     </row>
@@ -2150,12 +2440,22 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>número cuántico principal n, secundario l, magnético ml, spin ms, orbitales</t>
+          <t>número cuántico principal n, secundario l, magnético ml, spin ms, orbitales, números cuánticos como dirección electrón, piso departamento orientación, principal secundario magnético spin</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
           <t>Los 4 números cuánticos: principal (n), secundario (l), magnético (ml) y spin (ms)</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>números cuánticos como dirección electrón, piso departamento orientación, principal secundario magnético spin</t>
         </is>
       </c>
     </row>
@@ -2190,12 +2490,22 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>diamagnetismo, paramagnetismo, electrones desapareados, magnetismo, campo magnético</t>
+          <t>diamagnetismo, paramagnetismo, electrones desapareados, magnetismo, campo magnético, diamagnetismo paramagnetismo, electrones desapareados, comportamiento magnético orbitales</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
           <t>Diamagnetismo vs paramagnetismo: relación con electrones apareados y desapareados</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>diamagnetismo paramagnetismo, electrones desapareados, comportamiento magnético orbitales</t>
         </is>
       </c>
     </row>
@@ -2306,12 +2616,22 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>soluciones, introducción, soluto, solvente, disolvente, disolución, mezcla homogénea</t>
+          <t>soluciones, introducción, soluto, solvente, disolvente, disolución, mezcla homogénea, qué son soluciones, cómo se forman, componentes soluto solvente, preparación análisis</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
           <t>Conceptos básicos de soluciones: soluto, solvente, tipos de soluciones</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>qué son soluciones, cómo se forman, componentes soluto solvente, preparación análisis</t>
         </is>
       </c>
     </row>
@@ -2346,12 +2666,22 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>concentración porcentual, % m/m, % m/v, % v/v, porcentaje masa, volumen</t>
+          <t>concentración porcentual, % m/m, % m/v, % v/v, porcentaje masa, volumen, concentración porcentual %, masa/masa, masa/volumen, volumen/volumen, ejemplos cotidianos ejercicios examen</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
           <t>Concentraciones porcentuales: masa/masa, masa/volumen, volumen/volumen</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>concentración porcentual %, masa/masa, masa/volumen, volumen/volumen, ejemplos cotidianos ejercicios examen</t>
         </is>
       </c>
     </row>
@@ -2386,12 +2716,22 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>molaridad, M, moles por litro, concentración molar, mol/L</t>
+          <t>molaridad, M, moles por litro, concentración molar, mol/L, molaridad M, moles por litro, concentración molar</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
           <t>Molaridad: moles de soluto por litro de solución, cálculos y ejercicios</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>molaridad M, moles por litro, concentración molar</t>
         </is>
       </c>
     </row>
@@ -2426,12 +2766,22 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>normalidad, N, equivalentes, equivalente gramo, peso equivalente</t>
+          <t>normalidad, N, equivalentes, equivalente gramo, peso equivalente, normalidad N, equivalentes por litro, peso equivalente</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
           <t>Normalidad: número de equivalentes por litro de solución</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>normalidad N, equivalentes por litro, peso equivalente</t>
         </is>
       </c>
     </row>
@@ -2466,12 +2816,22 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>molalidad, m, moles por kg, concentración molal, solvente</t>
+          <t>molalidad, m, moles por kg, concentración molal, solvente, molalidad m, moles por kg solvente</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
           <t>Molalidad: moles de soluto por kilogramo de solvente</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>molalidad m, moles por kg solvente</t>
         </is>
       </c>
     </row>
@@ -2506,12 +2866,22 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>dilución, M1V1=M2V2, diluir, concentración, agregar solvente</t>
+          <t>dilución, M1V1=M2V2, diluir, concentración, agregar solvente, dilución M1V1=M2V2, agregar solvente, cálculos</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
           <t>Dilución de soluciones: fórmula M1V1 = M2V2, cálculos de dilución</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>dilución M1V1=M2V2, agregar solvente, cálculos</t>
         </is>
       </c>
     </row>
@@ -2546,12 +2916,22 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>fracción molar, Xi, moles, proporción, soluto, solvente</t>
+          <t>fracción molar, Xi, moles, proporción, soluto, solvente, fracción molar Xi, proporción moles componente total</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
           <t>Fracción molar: proporción de moles de un componente respecto al total</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>fracción molar Xi, proporción moles componente total</t>
         </is>
       </c>
     </row>
@@ -2622,12 +3002,22 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>precipitación, neutralización, redox, óxido-reducción, combinación, síntesis, descomposición, combustión, desplazamiento, desproporción, dismutación</t>
+          <t>precipitación, neutralización, redox, óxido-reducción, combinación, síntesis, descomposición, combustión, desplazamiento, desproporción, dismutación, todos tipos reacciones, precipitación neutralización redox combinación descomposición combustión desplazamiento desproporción</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
           <t>Todos los tipos de reacciones: precipitación, neutralización, redox, combinación, descomposición, combustión, desplazamiento simple/doble, desproporción</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>todos tipos reacciones, precipitación neutralización redox combinación descomposición combustión desplazamiento desproporción</t>
         </is>
       </c>
     </row>
@@ -2698,12 +3088,22 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>leyes de los gases, Boyle, Charles, Gay-Lussac, leyes combinadas, presión, volumen, temperatura</t>
+          <t>leyes de los gases, Boyle, Charles, Gay-Lussac, leyes combinadas, presión, volumen, temperatura, presión volumen temperatura gases, Boyle Charles Gay-Lussac leyes combinadas sentido físico</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
           <t>Leyes de los gases: Boyle (P×V), Charles (V/T), Gay-Lussac (P/T), ley combinada</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>presión volumen temperatura gases, Boyle Charles Gay-Lussac leyes combinadas sentido físico</t>
         </is>
       </c>
     </row>
@@ -2858,12 +3258,22 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Avogadro, volumen molar, 22.4L, STP, CNPT, moles y volumen</t>
+          <t>Avogadro, volumen molar, 22.4L, STP, CNPT, moles y volumen, volumen gas depende cantidad partículas, temperatura presión iguales, volumen molar</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
           <t>Ley de Avogadro: relación entre moles y volumen a condiciones estándar</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>volumen gas depende cantidad partículas, temperatura presión iguales, volumen molar</t>
         </is>
       </c>
     </row>
@@ -2938,12 +3348,22 @@
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>gas ideal, PV=nRT, ecuación de estado, R constante, presión volumen temperatura moles</t>
+          <t>gas ideal, PV=nRT, ecuación de estado, R constante, presión volumen temperatura moles, PV=nRT ecuación gases ideales, presión volumen temperatura moles R constante</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
           <t>Ecuación de los gases ideales PV = nRT: cálculos con presión, volumen, temperatura y moles</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>PV=nRT ecuación gases ideales, presión volumen temperatura moles R constante</t>
         </is>
       </c>
     </row>
@@ -3018,12 +3438,22 @@
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>estequiometría, gases, volumen molar, STP, reacciones con gases</t>
+          <t>estequiometría, gases, volumen molar, STP, reacciones con gases, estequiometría gases volumen molar STP reacciones con gases</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
           <t>Estequiometría aplicada a reacciones con gases usando volumen molar</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>estequiometría gases volumen molar STP reacciones con gases</t>
         </is>
       </c>
     </row>
@@ -3058,12 +3488,22 @@
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>fórmula mínima, fórmula molecular, gases, densidad, volumen molar</t>
+          <t>fórmula mínima, fórmula molecular, gases, densidad, volumen molar, fórmula mínima molecular gases densidad volumen molar</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
           <t>Determinación de fórmula mínima y molecular usando datos de gases</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>fórmula mínima molecular gases densidad volumen molar</t>
         </is>
       </c>
     </row>
@@ -3134,12 +3574,22 @@
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>electrolitos, no electrolitos, fuertes, débiles, conductividad, disociación, iones</t>
+          <t>electrolitos, no electrolitos, fuertes, débiles, conductividad, disociación, iones, electrolitos fuertes débiles no electrolitos, disociación iónica conductividad, ácidos fuertes bases sal</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
           <t>Electrolitos fuertes y débiles vs no electrolitos: disociación iónica y conductividad</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>electrolitos fuertes débiles no electrolitos, disociación iónica conductividad, ácidos fuertes bases sal</t>
         </is>
       </c>
     </row>
@@ -3210,12 +3660,22 @@
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>Arrhenius, Brønsted-Lowry, Lewis, ácido, base, protón, par electrónico</t>
+          <t>Arrhenius, Brønsted-Lowry, Lewis, ácido, base, protón, par electrónico, ácido base teorías, Arrhenius Brønsted-Lowry Lewis, sustancia comportamiento distinto</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
           <t>Teorías ácido-base: Arrhenius, Brønsted-Lowry y Lewis</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>ácido base teorías, Arrhenius Brønsted-Lowry Lewis, sustancia comportamiento distinto</t>
         </is>
       </c>
     </row>
@@ -3250,12 +3710,22 @@
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>pH, pOH, escala pH, ácido, neutro, básico, concentración H+, logaritmo</t>
+          <t>pH, pOH, escala pH, ácido, neutro, básico, concentración H+, logaritmo, escala pH, cálculo, concentración H+ OH-, ácido neutro básico logaritmo</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
           <t>Concepto de pH: escala, cálculo, relación con concentración de H+ y OH-</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>escala pH, cálculo, concentración H+ OH-, ácido neutro básico logaritmo</t>
         </is>
       </c>
     </row>
@@ -3290,12 +3760,22 @@
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>pH, soluciones, molaridad, dilución, cálculo pH en solución</t>
+          <t>pH, soluciones, molaridad, dilución, cálculo pH en solución, escala pH, cálculo, concentración H+ OH-, ácido neutro básico logaritmo</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
           <t>Cálculo de pH en soluciones: usando molaridad y volumen de ácidos/bases</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>escala pH, cálculo, concentración H+ OH-, ácido neutro básico logaritmo</t>
         </is>
       </c>
     </row>
@@ -3330,12 +3810,22 @@
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>Ka, Kb, pKa, pKb, constante de ionización, ácido débil, base débil, equilibrio</t>
+          <t>Ka, Kb, pKa, pKb, constante de ionización, ácido débil, base débil, equilibrio, Ka Kb pKa pKb, constante ionización, ácido débil base débil equilibrio</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
           <t>Constantes de ionización Ka y Kb, pKa y pKb: equilibrio de ácidos y bases débiles</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Ka Kb pKa pKb, constante ionización, ácido débil base débil equilibrio</t>
         </is>
       </c>
     </row>
@@ -3370,12 +3860,22 @@
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>buffer, tampón, amortiguador, Henderson-Hasselbalch, ácido débil + sal, pH estable</t>
+          <t>buffer, tampón, amortiguador, Henderson-Hasselbalch, ácido débil + sal, pH estable, buffer tampón amortiguador, Henderson-Hasselbalch, ácido débil + sal, pH estable</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
           <t>Soluciones buffer/tampón: ecuación de Henderson-Hasselbalch, preparación y funcionamiento</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>buffer tampón amortiguador, Henderson-Hasselbalch, ácido débil + sal, pH estable</t>
         </is>
       </c>
     </row>
@@ -3446,12 +3946,22 @@
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>enlace iónico, enlace covalente, enlace metálico, electronegatividad, transferencia, compartir</t>
+          <t>enlace iónico, enlace covalente, enlace metálico, electronegatividad, transferencia, compartir, enlaces químicos, iónico covalente metálico, características, cómo se forman, transferencia compartir electrones</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
           <t>Tipos de enlace: iónico (transferencia e-), covalente (compartir e-), metálico (mar de e-)</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>enlaces químicos, iónico covalente metálico, características, cómo se forman, transferencia compartir electrones</t>
         </is>
       </c>
     </row>
@@ -3486,12 +3996,22 @@
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>Lewis, estructura de puntos, pares enlazantes, pares libres, regla del octeto, electrones de valencia</t>
+          <t>Lewis, estructura de puntos, pares enlazantes, pares libres, regla del octeto, electrones de valencia, estructuras Lewis, electrones valencia, pares enlazantes libres, regla octeto</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
           <t>Estructuras de Lewis: representación de electrones de valencia, regla del octeto</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>estructuras Lewis, electrones valencia, pares enlazantes libres, regla octeto</t>
         </is>
       </c>
     </row>
@@ -3526,12 +4046,22 @@
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>polaridad, polar, apolar, momento dipolar, electronegatividad, enlace polar</t>
+          <t>polaridad, polar, apolar, momento dipolar, electronegatividad, enlace polar, polaridad enlaces moléculas, diferencia electronegatividad, momento dipolar</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
           <t>Polaridad de enlaces y moléculas: diferencia de electronegatividad, momento dipolar</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>polaridad enlaces moléculas, diferencia electronegatividad, momento dipolar</t>
         </is>
       </c>
     </row>
@@ -3566,12 +4096,22 @@
       </c>
       <c r="G79" s="3" t="inlineStr">
         <is>
-          <t>VSEPR, geometría molecular, geometría electrónica, lineal, trigonal, tetraédrica, angular</t>
+          <t>VSEPR, geometría molecular, geometría electrónica, lineal, trigonal, tetraédrica, angular, VSEPR, geometría molecular electrónica, lineal trigonal tetraédrica angular</t>
         </is>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
           <t>Geometría molecular y electrónica: teoría VSEPR, formas moleculares</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>VSEPR, geometría molecular electrónica, lineal trigonal tetraédrica angular</t>
         </is>
       </c>
     </row>
@@ -3606,12 +4146,22 @@
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>hibridación, sp, sp2, sp3, orbitales híbridos, mezcla de orbitales</t>
+          <t>hibridación, sp, sp2, sp3, orbitales híbridos, mezcla de orbitales, hibridación orbitales sp sp2 sp3, mezcla orbitales, predicción</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
           <t>Hibridación de orbitales: sp, sp², sp³, sp³d, sp³d² — predicción y ejemplos</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>hibridación orbitales sp sp2 sp3, mezcla orbitales, predicción</t>
         </is>
       </c>
     </row>
@@ -3646,12 +4196,22 @@
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>resonancia, estructuras resonantes, deslocalización, electrones, híbrido de resonancia</t>
+          <t>resonancia, estructuras resonantes, deslocalización, electrones, híbrido de resonancia, estructuras resonantes, deslocalización electrones, híbrido resonancia</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
           <t>Estructuras de resonancia: deslocalización de electrones, híbrido de resonancia</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>estructuras resonantes, deslocalización electrones, híbrido resonancia</t>
         </is>
       </c>
     </row>
@@ -3686,12 +4246,22 @@
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>orden de enlace, enlace simple, doble, triple, longitud, energía, fuerza</t>
+          <t>orden de enlace, enlace simple, doble, triple, longitud, energía, fuerza, orden enlace, simple doble triple, longitud energía fuerza</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
           <t>Orden de enlace: relación con longitud, energía y fuerza del enlace</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>orden enlace, simple doble triple, longitud energía fuerza</t>
         </is>
       </c>
     </row>
@@ -3762,12 +4332,22 @@
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>química orgánica, introducción, carbono, enlaces, cadenas, hibridación del carbono</t>
+          <t>química orgánica, introducción, carbono, enlaces, cadenas, hibridación del carbono, química orgánica carbono propiedades cadenas clasificación enlaces hibridación</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
           <t>Introducción a la orgánica: propiedades del carbono, tipos de cadenas, clasificación</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>química orgánica carbono propiedades cadenas clasificación enlaces hibridación</t>
         </is>
       </c>
     </row>
@@ -3802,12 +4382,22 @@
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>alcanos, alquenos, alquinos, enlace simple, doble, triple, saturados, insaturados, CnH2n+2</t>
+          <t>alcanos, alquenos, alquinos, enlace simple, doble, triple, saturados, insaturados, CnH2n+2, alcanos alquenos alquinos, enlace simple doble triple, saturados insaturados, nomenclatura IUPAC CnH2n+2</t>
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
           <t>Hidrocarburos: alcanos (enlace simple), alquenos (doble), alquinos (triple), nomenclatura IUPAC</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>alcanos alquenos alquinos, enlace simple doble triple, saturados insaturados, nomenclatura IUPAC CnH2n+2</t>
         </is>
       </c>
     </row>
@@ -3842,12 +4432,22 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>alcadienos, dienos, eninos, dobles enlaces, triple y doble enlace, nomenclatura</t>
+          <t>alcadienos, dienos, eninos, dobles enlaces, triple y doble enlace, nomenclatura, alcadienos dienos dobles enlaces eninos doble+triple enlace nomenclatura</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
           <t>Alcadienos (dos dobles enlaces) y eninos (doble + triple enlace): nomenclatura</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>alcadienos dienos dobles enlaces eninos doble+triple enlace nomenclatura</t>
         </is>
       </c>
     </row>
@@ -3882,12 +4482,22 @@
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>cicloalcanos, cicloalquenos, hidrocarburos cíclicos, anillos, nomenclatura</t>
+          <t>cicloalcanos, cicloalquenos, hidrocarburos cíclicos, anillos, nomenclatura, cicloalcanos cicloalquenos hidrocarburos cíclicos anillos nomenclatura propiedades</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
           <t>Hidrocarburos cíclicos: cicloalcanos, cicloalquenos, nomenclatura y propiedades</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>cicloalcanos cicloalquenos hidrocarburos cíclicos anillos nomenclatura propiedades</t>
         </is>
       </c>
     </row>
@@ -3922,12 +4532,22 @@
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>alcoholes, OH, grupo hidroxilo, primario, secundario, terciario, nomenclatura</t>
+          <t>alcoholes, OH, grupo hidroxilo, primario, secundario, terciario, nomenclatura, alcoholes grupo OH hidroxilo primario secundario terciario nomenclatura IUPAC propiedades</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
           <t>Alcoholes: grupo -OH, clasificación (1°, 2°, 3°), nomenclatura IUPAC</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>alcoholes grupo OH hidroxilo primario secundario terciario nomenclatura IUPAC propiedades</t>
         </is>
       </c>
     </row>
@@ -3962,12 +4582,22 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>ácidos carboxílicos, COOH, grupo carboxilo, nomenclatura, propiedades</t>
+          <t>ácidos carboxílicos, COOH, grupo carboxilo, nomenclatura, propiedades, ácidos carboxílicos grupo COOH carboxilo nomenclatura propiedades ácidas</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
           <t>Ácidos carboxílicos: grupo -COOH, nomenclatura, propiedades ácidas</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>ácidos carboxílicos grupo COOH carboxilo nomenclatura propiedades ácidas</t>
         </is>
       </c>
     </row>
@@ -4002,12 +4632,22 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>aldehídos, cetonas, grupo carbonilo, CHO, CO, nomenclatura</t>
+          <t>aldehídos, cetonas, grupo carbonilo, CHO, CO, nomenclatura, aldehídos cetonas grupo carbonilo C=O, aldehído extremo cadena mayor reactividad, cetonas cadena intermedia</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
           <t>Aldehídos (R-CHO) y cetonas (R-CO-R): grupo carbonilo, nomenclatura, diferencias</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>aldehídos cetonas grupo carbonilo C=O, aldehído extremo cadena mayor reactividad, cetonas cadena intermedia</t>
         </is>
       </c>
     </row>
@@ -4042,12 +4682,22 @@
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>ésteres, esterificación, RCOOR, grupo éster, nomenclatura</t>
+          <t>ésteres, esterificación, RCOOR, grupo éster, nomenclatura, ésteres esterificación RCOOR grupo éster nomenclatura propiedades</t>
         </is>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
           <t>Ésteres: formación por esterificación, nomenclatura, propiedades</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>ésteres esterificación RCOOR grupo éster nomenclatura propiedades</t>
         </is>
       </c>
     </row>
@@ -4082,12 +4732,22 @@
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>aminas, NH2, grupo amino, primaria, secundaria, terciaria, nomenclatura</t>
+          <t>aminas, NH2, grupo amino, primaria, secundaria, terciaria, nomenclatura, aminas derivados amoníaco, grupo funcional NH2, reemplazar hidrógeno grupos orgánicos</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
           <t>Aminas: grupo -NH₂, clasificación (1°, 2°, 3°), nomenclatura</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>aminas derivados amoníaco, grupo funcional NH2, reemplazar hidrógeno grupos orgánicos</t>
         </is>
       </c>
     </row>
@@ -4122,12 +4782,22 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>amidas, CONH2, enlace peptídico, nomenclatura, grupo amida</t>
+          <t>amidas, CONH2, enlace peptídico, nomenclatura, grupo amida, amidas grupo funcional CONH2, reacción ácidos carboxílicos aminas, enlace peptídico</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
           <t>Amidas: grupo -CONH₂, relación con enlace peptídico, nomenclatura</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>amidas grupo funcional CONH2, reacción ácidos carboxílicos aminas, enlace peptídico</t>
         </is>
       </c>
     </row>
@@ -4162,12 +4832,22 @@
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>éteres, R-O-R, grupo éter, nomenclatura, propiedades</t>
+          <t>éteres, R-O-R, grupo éter, nomenclatura, propiedades, éteres estructura R-O-R, diferenciar otros compuestos oxigenados, comportamiento químico</t>
         </is>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
           <t>Éteres: estructura R-O-R, nomenclatura IUPAC y común</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>éteres estructura R-O-R, diferenciar otros compuestos oxigenados, comportamiento químico</t>
         </is>
       </c>
     </row>
@@ -4202,12 +4882,22 @@
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>benceno, aromáticos, anillo bencénico, sustitución, nomenclatura, arenos</t>
+          <t>benceno, aromáticos, anillo bencénico, sustitución, nomenclatura, arenos, sin contenido texto, solo título</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
           <t>Compuestos aromáticos: benceno, nomenclatura de derivados, reacciones de sustitución</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>sin contenido texto, solo título</t>
         </is>
       </c>
     </row>
@@ -4242,12 +4932,22 @@
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>haluros de alquilo, R-X, flúor, cloro, bromo, yodo, halogenación, nomenclatura</t>
+          <t>haluros de alquilo, R-X, flúor, cloro, bromo, yodo, halogenación, nomenclatura, haluros alquilo R-X flúor cloro bromo yodo, clasificación primario secundario terciario</t>
         </is>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
           <t>Haluros de alquilo: R-X (F, Cl, Br, I), nomenclatura y clasificación</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>haluros alquilo R-X flúor cloro bromo yodo, clasificación primario secundario terciario</t>
         </is>
       </c>
     </row>
@@ -4282,12 +4982,22 @@
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>reacciones orgánicas, sustitución, eliminación, adición, oxidación, reducción, SN1, SN2, E1, E2</t>
+          <t>reacciones orgánicas, sustitución, eliminación, adición, oxidación, reducción, SN1, SN2, E1, E2, reacciones orgánicas, sustitución eliminación adición oxidación reducción</t>
         </is>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
           <t>Tipos de reacciones orgánicas: sustitución, eliminación, adición, oxidación, reducción</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>reacciones orgánicas, sustitución eliminación adición oxidación reducción</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar curso Biología UCV al chatbot
Chatbot ahora cubre Química UCV (96 registros) y Biología UCV (41 registros).
Interfaz actualizada: título, sidebar con ambos cursos, sugerencias mixtas.
</commit_message>
<xml_diff>
--- a/quimica_ucv_base_datos.xlsx
+++ b/quimica_ucv_base_datos.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Base de Datos Química UCV" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Base de Datos Biología UCV" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,8 +46,13 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +69,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D4E6F1"/>
         <bgColor rgb="00D4E6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B5E20"/>
+        <bgColor rgb="001B5E20"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
   </fills>
@@ -84,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -99,6 +117,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J97"/>
+  <dimension ref="A1:K97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -528,6 +552,11 @@
           <t>Contenido Real Verificado</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -564,6 +593,11 @@
           <t>Lección introductoria sobre los fundamentos generales de la química: conceptos de materia y energía</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -614,6 +648,11 @@
           <t>conceptos básicos química, materia energía, propiedades, clasificación, estados materia, sustancias puras mezclas, h5p interactivo</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -650,6 +689,11 @@
           <t>Lección sobre formulación y nomenclatura de compuestos inorgánicos: óxidos, hidróxidos, ácidos, sales</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -700,6 +744,11 @@
           <t>formular nombrar compuestos oxigenados, óxidos básicos ácidos anhídridos, nomenclatura IUPAC stock tradicional números oxidación</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -750,6 +799,11 @@
           <t>formular nombrar compuestos hidrogenados, hidruros metálicos, hidrógeno combinado otros elementos</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -800,6 +854,11 @@
           <t>formular nombrar sales binarias, metal + no metal, sin oxígeno, números oxidación intercambio</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -850,6 +909,11 @@
           <t>formular nombrar hidróxidos, metal + grupo hidroxilo OH, números oxidación intercambio valencias</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -900,6 +964,11 @@
           <t>formular nombrar ácidos oxácidos, hidrógeno oxígeno no metal, números oxidación reglas formulación</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -950,6 +1019,11 @@
           <t>formular nombrar sales neutras oxisales, neutralización total ácido base, catión anión</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1000,6 +1074,11 @@
           <t>sales ácidas neutralización parcial, hidrógeno restante bisales</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1050,6 +1129,11 @@
           <t>sales básicas hidroxisales, neutralización parcial bases, grupo OH restante</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1086,6 +1170,11 @@
           <t>Lección sobre cálculo de peso/masa molecular de compuestos químicos</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1136,6 +1225,11 @@
           <t>cálculo peso molecular usando tabla periódica, suma masas atómicas, uma, dalton</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1172,6 +1266,11 @@
           <t>Lección sobre relaciones entre átomos, moléculas, moles y gramos. Número de Avogadro</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1222,6 +1321,11 @@
           <t>conversiones moles átomos gramos, número Avogadro 6.022x10^23</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1272,6 +1376,11 @@
           <t>cómo está formada materia átomos, iones, unidades más pequeñas elementos, ganar perder electrones</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -1312,6 +1421,11 @@
           <t>Cuestionario/simulación interactiva sobre formación de átomos</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1362,6 +1476,11 @@
           <t>conversión directa átomos gramos, combinar Avogadro masa molar</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1412,6 +1531,11 @@
           <t>concepto molécula, conversiones moles número moléculas, Avogadro</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1448,6 +1572,11 @@
           <t>Lección sobre cálculo de composición porcentual o centesimal de compuestos</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1498,6 +1627,11 @@
           <t>calcular composición centesimal porcentual paso a paso, porcentajes ejercicios</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1534,6 +1668,11 @@
           <t>Lección sobre determinación de fórmula mínima (empírica) y fórmula molecular</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1584,6 +1723,11 @@
           <t>fórmula mínima molecular gases densidad volumen molar</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1634,6 +1778,11 @@
           <t>fórmula mínima empírica, proporción mínima moles simplificar datos composición</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1670,6 +1819,11 @@
           <t>Lección completa sobre estequiometría: cálculos basados en ecuaciones químicas balanceadas</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1720,6 +1874,11 @@
           <t>video estequiometría, balanceo ecuaciones químicas, relaciones molares, coeficientes</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1770,6 +1929,11 @@
           <t>identificar reactivo limitante exceso, cálculo rendimiento teórico, cantidad producto</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -1810,6 +1974,11 @@
           <t>Ejercicios explicados paso a paso sobre reactivo limitante y en exceso</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -1860,6 +2029,11 @@
           <t>rendimiento porcentual real teórico eficiencia reacción</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -1910,6 +2084,11 @@
           <t>estequiometría soluciones molaridad volumen reacciones en solución</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -1960,6 +2139,11 @@
           <t>fórmula mínima empírica, proporción mínima moles simplificar datos composición</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1996,6 +2180,11 @@
           <t>Lección sobre estructura del átomo y propiedades periódicas de los elementos</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -2046,6 +2235,11 @@
           <t>video sobre radio atómico radio iónico energía ionización tendencias periódicas</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -2086,6 +2280,11 @@
           <t>Cuestionario evaluativo sobre radio atómico y radio iónico</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -2136,6 +2335,11 @@
           <t>diferenciar afinidad electrónica electronegatividad, propiedades periódicas, cómo átomos atraen electrones, variación tabla periódica</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -2186,6 +2390,11 @@
           <t>clasificación especies, isótopos mismo Z, isóbaros mismo A, isótonos mismo N, isoelectrónicos</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -2236,6 +2445,11 @@
           <t>cálculo masa atómica promedio, abundancia isotópica porcentaje natural</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2272,6 +2486,11 @@
           <t>Lección sobre configuración electrónica de los elementos: principios y reglas</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -2322,6 +2541,11 @@
           <t>configuración electrónica, Aufbau, Hund, Pauli, subniveles s p d f, Moeller</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -2372,6 +2596,11 @@
           <t>configuración electrónica, Aufbau, Hund, Pauli, subniveles s p d f, Moeller</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2408,6 +2637,11 @@
           <t>Lección sobre los cuatro números cuánticos que describen el estado de un electrón</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -2458,6 +2692,11 @@
           <t>números cuánticos como dirección electrón, piso departamento orientación, principal secundario magnético spin</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -2508,6 +2747,11 @@
           <t>diamagnetismo paramagnetismo, electrones desapareados, comportamiento magnético orbitales</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -2548,6 +2792,11 @@
           <t>Cuestionario evaluativo sobre números cuánticos</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2584,6 +2833,11 @@
           <t>Lección completa sobre soluciones: tipos de concentración y cálculos</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -2634,6 +2888,11 @@
           <t>qué son soluciones, cómo se forman, componentes soluto solvente, preparación análisis</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -2684,6 +2943,11 @@
           <t>concentración porcentual %, masa/masa, masa/volumen, volumen/volumen, ejemplos cotidianos ejercicios examen</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -2734,6 +2998,11 @@
           <t>molaridad M, moles por litro, concentración molar</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
@@ -2784,6 +3053,11 @@
           <t>normalidad N, equivalentes por litro, peso equivalente</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -2834,6 +3108,11 @@
           <t>molalidad m, moles por kg solvente</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -2884,6 +3163,11 @@
           <t>dilución M1V1=M2V2, agregar solvente, cálculos</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -2934,6 +3218,11 @@
           <t>fracción molar Xi, proporción moles componente total</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2970,6 +3259,11 @@
           <t>Lección sobre clasificación de las reacciones químicas</t>
         </is>
       </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
@@ -3020,6 +3314,11 @@
           <t>todos tipos reacciones, precipitación neutralización redox combinación descomposición combustión desplazamiento desproporción</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3056,6 +3355,11 @@
           <t>Lección completa sobre gases: leyes, ecuación de gas ideal, estequiometría</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -3106,6 +3410,11 @@
           <t>presión volumen temperatura gases, Boyle Charles Gay-Lussac leyes combinadas sentido físico</t>
         </is>
       </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n">
@@ -3146,6 +3455,11 @@
           <t>Ejercicios explicados sobre la ley de Charles (V1/T1 = V2/T2)</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -3186,6 +3500,11 @@
           <t>Ejercicios explicados sobre la ley de Boyle (P1V1 = P2V2)</t>
         </is>
       </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">
@@ -3226,6 +3545,11 @@
           <t>Ejercicios explicados sobre leyes combinadas de los gases</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -3276,6 +3600,11 @@
           <t>volumen gas depende cantidad partículas, temperatura presión iguales, volumen molar</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n">
@@ -3316,6 +3645,11 @@
           <t>Ejercicios explicados sobre la ley de Avogadro</t>
         </is>
       </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -3366,6 +3700,11 @@
           <t>PV=nRT ecuación gases ideales, presión volumen temperatura moles R constante</t>
         </is>
       </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
@@ -3406,6 +3745,11 @@
           <t>Cuestionario evaluativo sobre ecuación de gases ideales</t>
         </is>
       </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -3456,6 +3800,11 @@
           <t>estequiometría gases volumen molar STP reacciones con gases</t>
         </is>
       </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
@@ -3506,6 +3855,11 @@
           <t>fórmula mínima molecular gases densidad volumen molar</t>
         </is>
       </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3542,6 +3896,11 @@
           <t>Lección sobre propiedades electrolíticas de las soluciones</t>
         </is>
       </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
@@ -3592,6 +3951,11 @@
           <t>electrolitos fuertes débiles no electrolitos, disociación iónica conductividad, ácidos fuertes bases sal</t>
         </is>
       </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -3628,6 +3992,11 @@
           <t>Lección completa sobre teoría ácido-base, pH y soluciones buffer</t>
         </is>
       </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
@@ -3678,6 +4047,11 @@
           <t>ácido base teorías, Arrhenius Brønsted-Lowry Lewis, sustancia comportamiento distinto</t>
         </is>
       </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
@@ -3728,6 +4102,11 @@
           <t>escala pH, cálculo, concentración H+ OH-, ácido neutro básico logaritmo</t>
         </is>
       </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -3778,6 +4157,11 @@
           <t>escala pH, cálculo, concentración H+ OH-, ácido neutro básico logaritmo</t>
         </is>
       </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
@@ -3828,6 +4212,11 @@
           <t>Ka Kb pKa pKb, constante ionización, ácido débil base débil equilibrio</t>
         </is>
       </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -3878,6 +4267,11 @@
           <t>buffer tampón amortiguador, Henderson-Hasselbalch, ácido débil + sal, pH estable</t>
         </is>
       </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -3914,6 +4308,11 @@
           <t>Lección completa sobre enlaces químicos: tipos, Lewis, geometría, hibridación</t>
         </is>
       </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -3964,6 +4363,11 @@
           <t>enlaces químicos, iónico covalente metálico, características, cómo se forman, transferencia compartir electrones</t>
         </is>
       </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
@@ -4014,6 +4418,11 @@
           <t>estructuras Lewis, electrones valencia, pares enlazantes libres, regla octeto</t>
         </is>
       </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
@@ -4064,6 +4473,11 @@
           <t>polaridad enlaces moléculas, diferencia electronegatividad, momento dipolar</t>
         </is>
       </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
@@ -4114,6 +4528,11 @@
           <t>VSEPR, geometría molecular electrónica, lineal trigonal tetraédrica angular</t>
         </is>
       </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -4164,6 +4583,11 @@
           <t>hibridación orbitales sp sp2 sp3, mezcla orbitales, predicción</t>
         </is>
       </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
@@ -4214,6 +4638,11 @@
           <t>estructuras resonantes, deslocalización electrones, híbrido resonancia</t>
         </is>
       </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n">
@@ -4264,6 +4693,11 @@
           <t>orden enlace, simple doble triple, longitud energía fuerza</t>
         </is>
       </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -4300,6 +4734,11 @@
           <t>Lección completa sobre química orgánica: hidrocarburos y grupos funcionales</t>
         </is>
       </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n">
@@ -4350,6 +4789,11 @@
           <t>química orgánica carbono propiedades cadenas clasificación enlaces hibridación</t>
         </is>
       </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -4400,6 +4844,11 @@
           <t>alcanos alquenos alquinos, enlace simple doble triple, saturados insaturados, nomenclatura IUPAC CnH2n+2</t>
         </is>
       </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
@@ -4450,6 +4899,11 @@
           <t>alcadienos dienos dobles enlaces eninos doble+triple enlace nomenclatura</t>
         </is>
       </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
@@ -4500,6 +4954,11 @@
           <t>cicloalcanos cicloalquenos hidrocarburos cíclicos anillos nomenclatura propiedades</t>
         </is>
       </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
@@ -4550,6 +5009,11 @@
           <t>alcoholes grupo OH hidroxilo primario secundario terciario nomenclatura IUPAC propiedades</t>
         </is>
       </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n">
@@ -4600,6 +5064,11 @@
           <t>ácidos carboxílicos grupo COOH carboxilo nomenclatura propiedades ácidas</t>
         </is>
       </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n">
@@ -4650,6 +5119,11 @@
           <t>aldehídos cetonas grupo carbonilo C=O, aldehído extremo cadena mayor reactividad, cetonas cadena intermedia</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n">
@@ -4700,6 +5174,11 @@
           <t>ésteres esterificación RCOOR grupo éster nomenclatura propiedades</t>
         </is>
       </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n">
@@ -4750,6 +5229,11 @@
           <t>aminas derivados amoníaco, grupo funcional NH2, reemplazar hidrógeno grupos orgánicos</t>
         </is>
       </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n">
@@ -4800,6 +5284,11 @@
           <t>amidas grupo funcional CONH2, reacción ácidos carboxílicos aminas, enlace peptídico</t>
         </is>
       </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n">
@@ -4850,6 +5339,11 @@
           <t>éteres estructura R-O-R, diferenciar otros compuestos oxigenados, comportamiento químico</t>
         </is>
       </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
@@ -4900,6 +5394,11 @@
           <t>sin contenido texto, solo título</t>
         </is>
       </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n">
@@ -4950,6 +5449,11 @@
           <t>haluros alquilo R-X flúor cloro bromo yodo, clasificación primario secundario terciario</t>
         </is>
       </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
@@ -4998,6 +5502,11 @@
       <c r="J97" t="inlineStr">
         <is>
           <t>reacciones orgánicas, sustitución eliminación adición oxidación reducción</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Química UCV</t>
         </is>
       </c>
     </row>
@@ -5144,4 +5653,1877 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Tema/Subtema</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Nombre Completo</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Palabras Clave</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Descripción para IA</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr"/>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/una-vision-de-la-vida/</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>visión vida, biología celular, seres vivos, evolución, taxonomía, origen vida</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Lección introductoria sobre biología: características de los seres vivos, evolución, taxonomía y origen de la vida</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Características de los Seres Vivos</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida &gt; Características de los Seres Vivos</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/una-vision-de-la-vida/topics/caracteristicas-de-los-seres-vivos/</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>características seres vivos, organización celular, nutrición, metabolismo, crecimiento, reproducción, respuesta estímulos, homeostasis, adaptación</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Principales características que permiten reconocer los seres vivos: organización celular, nutrición, metabolismo, crecimiento, reproducción, respuesta a estímulos</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Evolución</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida &gt; Evolución</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/una-vision-de-la-vida/topics/evolucion/</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>evolución, selección natural, Darwin, adaptación, especiación, cambio especies, herencia, variación genética</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Conceptos de evolución biológica: selección natural, adaptación, especiación y cambio en las especies</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Tipología Celular</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida &gt; Tipología Celular</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/una-vision-de-la-vida/topics/tipologia-celular/</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>tipología celular, célula procariota, célula eucariota, célula animal, célula vegetal, organelos, diferencias</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Tipos de células: procariotas y eucariotas, células animales y vegetales, organelos y diferencias</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Taxonomía</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida &gt; Taxonomía</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/una-vision-de-la-vida/topics/taxonomia/</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>taxonomía, clasificación seres vivos, reinos, dominios, Linneo, nomenclatura binomial, filogenia, árbol vida</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Clasificación de los seres vivos: reinos, dominios, nomenclatura binomial de Linneo</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Niveles de Organización Biológica</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida &gt; Niveles de Organización Biológica</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/una-vision-de-la-vida/topics/niveles-de-organizacion-biologica/</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>niveles organización, átomo, molécula, célula, tejido, órgano, sistema, organismo, población, comunidad, ecosistema, biósfera</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Niveles de organización biológica: desde átomo hasta biósfera</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Micoplasmas, Virus e Historia de la Biología</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida &gt; Micoplasmas, Virus e Historia de la Biología</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/una-vision-de-la-vida/topics/micoplasmas-virus-e-historia-de-la-biologia/</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>micoplasmas, virus, historia biología, microorganismos, patógenos, virología, bacterias pequeñas</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Micoplasmas y virus: estructura, características y su lugar en la historia de la biología</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Método de Investigación Científica</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida &gt; Método de Investigación Científica</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/una-vision-de-la-vida/topics/metodo-de-investigacion-cientifica/</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>método científico, investigación, observación, hipótesis, experimentación, conclusión, variables, pasos método científico</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Pasos del método de investigación científica: observación, planteamiento del problema, hipótesis, experimentación, conclusión</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Teorías Del Origen de la Vida</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Una Visión De la Vida &gt; Teorías Del Origen de la Vida</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/una-vision-de-la-vida/topics/teorias-del-origen-de-la-vida/</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>origen vida, generación espontánea, biogénesis, panspermia, sopa primordial, Oparin, Miller, abiogénesis</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Teorías sobre el origen de la vida: generación espontánea, biogénesis, panspermia, sopa primordial de Oparin</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Biomoléculas Inorgánicas</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Biomoléculas Inorgánicas</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-inorganicas/</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>biomoléculas inorgánicas, agua, minerales, sales, biología molecular</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre biomoléculas inorgánicas: el agua y su importancia en los procesos biológicos</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Inorgánicas</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Agua Parte 1</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Inorgánicas &gt; Agua Parte 1</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-inorganicas/topics/agua-parte-1/</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>agua, biomolécula inorgánica, estructura molecular, propiedades agua, puente hidrógeno, polaridad, solvente universal</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Importancia del agua como biomolécula: estructura molecular, propiedades, puentes de hidrógeno</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Inorgánicas</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Agua Parte 2</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Inorgánicas &gt; Agua Parte 2</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-inorganicas/topics/agua-parte-2/</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>agua parte 2, propiedades agua, procesos biológicos, capilaridad, tensión superficial, calor específico, ionización agua</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Propiedades del agua y su importancia en procesos biológicos: capilaridad, tensión superficial, calor específico</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>biomoléculas orgánicas, carbohidratos, lípidos, proteínas, ácidos nucleicos, enzimas, vitaminas</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre biomoléculas orgánicas: carbohidratos, lípidos, proteínas, ácidos nucleicos, enzimas y vitaminas</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Carbohidratos Parte 1</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Carbohidratos Parte 1</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/carbohidratos-parte-1/</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>carbohidratos, glúcidos, azúcares, monosacáridos, glucosa, fructosa, galactosa, composición, clasificación</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Carbohidratos como biomoléculas orgánicas: composición, clasificación, monosacáridos</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Carbohidratos Parte 2</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Carbohidratos Parte 2</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/carbohidratos-parte-2/</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>carbohidratos parte 2, disacáridos, oligosacáridos, sacarosa, lactosa, maltosa, enlace glucosídico</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Disacáridos y oligosacáridos: sacarosa, lactosa, maltosa, enlace glucosídico</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Carbohidratos Parte 3</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Carbohidratos Parte 3</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/carbohidratos-parte-3/</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>carbohidratos parte 3, polisacáridos, almidón, glucógeno, celulosa, quitina, funciones</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Polisacáridos: almidón, glucógeno, celulosa, quitina y sus funciones biológicas</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Lípidos Parte 1</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Lípidos Parte 1</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/lipidos-parte-1/</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>lípidos, grasas, aceites, ácidos grasos, saturados, insaturados, triglicéridos, clasificación</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Lípidos: clasificación, ácidos grasos saturados e insaturados, triglicéridos</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Lípidos Parte 2</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Lípidos Parte 2</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/lipidos-parte-2/</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>lípidos parte 2, fosfolípidos, membrana celular, esteroides, colesterol, ceras</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Fosfolípidos, membrana celular, esteroides, colesterol y ceras</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Lípidos Parte 3</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Lípidos Parte 3</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/lipidos-parte-3/</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>lípidos parte 3, funciones lípidos, energía, aislamiento, protección, hormonas esteroideas</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Funciones de los lípidos: reserva energética, aislamiento, protección, hormonas esteroideas</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Aminoácidos Péptidos Proteínas</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Aminoácidos Péptidos Proteínas</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/aminoacidos-peptidos-proteinas/</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>aminoácidos, péptidos, proteínas, enlace peptídico, estructura primaria, secundaria, terciaria, cuaternaria, desnaturalización</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Aminoácidos, péptidos y proteínas: enlace peptídico, niveles estructurales, desnaturalización</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Ácido Nucleico</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Ácido Nucleico</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/acido-nucleico/</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>ácido nucleico, ADN, ARN, nucleótidos, bases nitrogenadas, adenina, guanina, citosina, timina, uracilo, doble hélice</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Ácidos nucleicos: ADN y ARN, nucleótidos, bases nitrogenadas, estructura de doble hélice</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Enzima</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Enzima</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/enzima/</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>enzimas, catalizador biológico, sustrato, sitio activo, cofactor, coenzima, inhibición, cinética enzimática</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Enzimas como catalizadores biológicos: sustrato, sitio activo, cofactores, inhibición enzimática</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Vitaminas</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Biomoléculas Orgánicas &gt; Vitaminas</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/biomoleculas-organicas/topics/vitaminas/</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>vitaminas, hidrosolubles, liposolubles, vitamina A, B, C, D, E, K, deficiencia, función</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Vitaminas hidrosolubles y liposolubles: clasificación, funciones y deficiencias</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Membranas Biológicas</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr"/>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Membranas Biológicas</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/membranas-biologicas/</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>membranas biológicas, membrana celular, bicapa lipídica, transporte</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre membranas biológicas: estructura, función y transporte celular</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Membranas Biológicas</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Membranas Biológicas Parte 1</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Membranas Biológicas &gt; Membranas Biológicas Parte 1</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/membranas-biologicas/topics/membranas-biologicas-parte-1/</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>membrana celular, bicapa lipídica, modelo mosaico fluido, fosfolípidos, proteínas membrana, permeabilidad selectiva</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Estructura de la membrana celular: bicapa lipídica, modelo mosaico fluido, proteínas de membrana</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Membranas Biológicas</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Membranas Biológicas Parte 2</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Membranas Biológicas &gt; Membranas Biológicas Parte 2</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/membranas-biologicas/topics/membranas-biologicas-parte-2/</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>transporte celular, difusión, ósmosis, transporte activo, pasivo, endocitosis, exocitosis, bomba sodio potasio</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Transporte celular: difusión, ósmosis, transporte activo y pasivo, endocitosis, exocitosis</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Organización de la Célula</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr"/>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Organización de la Célula</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/organizacion-de-la-celula/</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>organización célula, organelos, endomembranas, citoesqueleto</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre la organización interna de la célula: sistema de endomembranas y citoesqueleto</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Organización de la Célula</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Sistema de Endomembranas</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Organización de la Célula &gt; Sistema de Endomembranas</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/organizacion-de-la-celula/topics/sistema-de-endomembranas/</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>sistema endomembranas, retículo endoplásmico, aparato Golgi, lisosomas, vesículas, RE liso, RE rugoso</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Sistema de endomembranas: retículo endoplásmico liso y rugoso, aparato de Golgi, lisosomas</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Organización de la Célula</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Citoesqueleto</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Organización de la Célula &gt; Citoesqueleto</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/organizacion-de-la-celula/topics/citoesqueleto/</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>citoesqueleto, microtúbulos, microfilamentos, filamentos intermedios, movimiento celular, forma célula</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Citoesqueleto: microtúbulos, microfilamentos, filamentos intermedios y su función en la célula</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Producción de Energía y Respiración</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr"/>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Producción de Energía y Respiración</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/produccion-de-energia-y-respiracion/</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>producción energía, respiración celular, mitocondrias, ATP</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre producción de energía celular y respiración</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Producción de Energía y Respiración</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Mitocondrias</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Producción de Energía y Respiración &gt; Mitocondrias</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/produccion-de-energia-y-respiracion/topics/mitocondrias/</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>mitocondrias, respiración celular, ATP, glucólisis, ciclo Krebs, cadena transporte electrones, fosforilación oxidativa</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Mitocondrias y respiración celular: glucólisis, ciclo de Krebs, cadena de transporte de electrones, producción de ATP</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Fotosíntesis</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr"/>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Fotosíntesis</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/fotosintesis/</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>fotosíntesis, cloroplasto, luz, energía solar</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre fotosíntesis</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Fotosíntesis</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Fotosíntesis</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Fotosíntesis &gt; Fotosíntesis</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/fotosintesis/topics/fotosintesis/</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>fotosíntesis, cloroplasto, clorofila, fase luminosa, fase oscura, ciclo Calvin, CO2, O2, glucosa, tilacoides, estroma</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Fotosíntesis: cloroplasto, clorofila, fase luminosa, ciclo de Calvin, producción de glucosa y oxígeno</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Microscopía</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr"/>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Microscopía</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/microscopia/</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>microscopía, microscopio, observación células</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre microscopía</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Microscopía</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Microscopía</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Microscopía &gt; Microscopía</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/microscopia/topics/microscopia/</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>microscopio, microscopía óptica, electrónica, resolución, aumento, preparación muestras, tinción, tipos microscopio</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Microscopía: tipos de microscopio (óptico, electrónico), resolución, aumento, preparación de muestras</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>División Celular</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr"/>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>División Celular</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/division-celular/</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>división celular, mitosis, meiosis, ciclo celular</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre división celular: mitosis y meiosis</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>División Celular</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Mitosis y Meiosis</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>División Celular &gt; Mitosis y Meiosis</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/division-celular/topics/mitosis-y-meiosis/</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>mitosis, meiosis, ciclo celular, profase, metafase, anafase, telofase, cromosomas, diploide, haploide, crossing over, gametos</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Mitosis y meiosis: fases, diferencias, cromosomas, crossing over, formación de gametos</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Histología</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr"/>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Histología</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/histologia/</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>histología, tejidos, clasificación tejidos</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre histología y tipos de tejidos</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Histología</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Tejidos</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Histología &gt; Tejidos</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/histologia/topics/tejidos/</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>tejidos, epitelial, conectivo, muscular, nervioso, histología, clasificación tejidos, funciones</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Tipos de tejidos: epitelial, conectivo, muscular y nervioso, clasificación y funciones</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Continuidad de la Vida</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr"/>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Continuidad de la Vida</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/continuidad-de-la-vida/</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>continuidad vida, genética, herencia</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Lección sobre genética y continuidad de la vida</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Continuidad de la Vida</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Genética</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Continuidad de la Vida &gt; Genética</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fundamentos-de-biologia-general/lessons/continuidad-de-la-vida/topics/genetica/</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>genética, Mendel, leyes herencia, dominante, recesivo, genotipo, fenotipo, alelos, homocigoto, heterocigoto, Punnett, herencia ligada sexo</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Genética: leyes de Mendel, dominancia, genotipo, fenotipo, cuadro de Punnett, herencia ligada al sexo</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Biología UCV</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Enriquecer keywords de Biología UCV con contenido real de WordPress
29 temas actualizados con contenido verificado. Precisión Biología sube de ~75% a ~90%.
</commit_message>
<xml_diff>
--- a/quimica_ucv_base_datos.xlsx
+++ b/quimica_ucv_base_datos.xlsx
@@ -5794,7 +5794,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>características seres vivos, organización celular, nutrición, metabolismo, crecimiento, reproducción, respuesta estímulos, homeostasis, adaptación</t>
+          <t>características seres vivos, organización celular, nutrición, metabolismo, crecimiento, reproducción, respuesta estímulos, homeostasis, adaptación, organización celular, nutrición, metabolismo, crecimiento, reproducción, respuesta estímulos, adaptación, capacidad evolucionar</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -5839,7 +5839,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>evolución, selección natural, Darwin, adaptación, especiación, cambio especies, herencia, variación genética</t>
+          <t>evolución, selección natural, Darwin, adaptación, especiación, cambio especies, herencia, variación genética, células cambiando perfeccionándose, origen primeras formas celulares, procariotas eucariotas, evolución celular, tiempo geológico</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>tipología celular, célula procariota, célula eucariota, célula animal, célula vegetal, organelos, diferencias</t>
+          <t>tipología celular, célula procariota, célula eucariota, célula animal, célula vegetal, organelos, diferencias, clasificación células, procariotas eucariotas, células animales vegetales, bacterianas, fúngicas, características estructurales funcionales</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>taxonomía, clasificación seres vivos, reinos, dominios, Linneo, nomenclatura binomial, filogenia, árbol vida</t>
+          <t>taxonomía, clasificación seres vivos, reinos, dominios, Linneo, nomenclatura binomial, filogenia, árbol vida, clasificación seres vivos, dominio reino filo clase orden familia género especie, relaciones evolutivas, categorías taxonómicas</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>niveles organización, átomo, molécula, célula, tejido, órgano, sistema, organismo, población, comunidad, ecosistema, biósfera</t>
+          <t>niveles organización, átomo, molécula, célula, tejido, órgano, sistema, organismo, población, comunidad, ecosistema, biósfera, organización vida, estructuras simples complejas, célula tejido órgano sistema organismo, niveles biológicos</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>micoplasmas, virus, historia biología, microorganismos, patógenos, virología, bacterias pequeñas</t>
+          <t>micoplasmas, virus, historia biología, microorganismos, patógenos, virología, bacterias pequeñas, micoplasmas bacterias pequeñas, virus estructura replicación, historia biología, microscopio descubrimiento célula</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>método científico, investigación, observación, hipótesis, experimentación, conclusión, variables, pasos método científico</t>
+          <t>método científico, investigación, observación, hipótesis, experimentación, conclusión, variables, pasos método científico, pasos investigación científica, observación problema hipótesis experimentación conclusión, variables, método científico ordenado confiable</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -6109,7 +6109,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>origen vida, generación espontánea, biogénesis, panspermia, sopa primordial, Oparin, Miller, abiogénesis</t>
+          <t>origen vida, generación espontánea, biogénesis, panspermia, sopa primordial, Oparin, Miller, abiogénesis, origen vida Tierra, generación espontánea, biogénesis, panspermia, sopa primordial Oparin, experimento Miller</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -6195,7 +6195,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>agua, biomolécula inorgánica, estructura molecular, propiedades agua, puente hidrógeno, polaridad, solvente universal</t>
+          <t>agua, biomolécula inorgánica, estructura molecular, propiedades agua, puente hidrógeno, polaridad, solvente universal, agua biomolécula inorgánica, estructura molecular, propiedades, puente hidrógeno, polaridad, solvente universal, importancia vida</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>agua parte 2, propiedades agua, procesos biológicos, capilaridad, tensión superficial, calor específico, ionización agua</t>
+          <t>agua parte 2, propiedades agua, procesos biológicos, capilaridad, tensión superficial, calor específico, ionización agua, propiedades agua procesos biológicos, capilaridad, tensión superficial, calor específico, ionización agua, pH</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>carbohidratos, glúcidos, azúcares, monosacáridos, glucosa, fructosa, galactosa, composición, clasificación</t>
+          <t>carbohidratos, glúcidos, azúcares, monosacáridos, glucosa, fructosa, galactosa, composición, clasificación, carbohidratos biomoléculas orgánicas, composición química, clasificación, monosacáridos disacáridos polisacáridos, glucosa fructosa</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>carbohidratos parte 2, disacáridos, oligosacáridos, sacarosa, lactosa, maltosa, enlace glucosídico</t>
+          <t>carbohidratos parte 2, disacáridos, oligosacáridos, sacarosa, lactosa, maltosa, enlace glucosídico, disacáridos oligosacáridos, sacarosa lactosa maltosa, enlace glucosídico, estructura ciclación</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>carbohidratos parte 3, polisacáridos, almidón, glucógeno, celulosa, quitina, funciones</t>
+          <t>carbohidratos parte 3, polisacáridos, almidón, glucógeno, celulosa, quitina, funciones, polisacáridos, almidón glucógeno celulosa quitina, funciones biológicas, reserva energética estructura</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -6461,7 +6461,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>lípidos, grasas, aceites, ácidos grasos, saturados, insaturados, triglicéridos, clasificación</t>
+          <t>lípidos, grasas, aceites, ácidos grasos, saturados, insaturados, triglicéridos, clasificación, lípidos grasas aceites, ácidos grasos saturados insaturados, triglicéridos, clasificación estructura</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -6506,7 +6506,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>lípidos parte 2, fosfolípidos, membrana celular, esteroides, colesterol, ceras</t>
+          <t>lípidos parte 2, fosfolípidos, membrana celular, esteroides, colesterol, ceras, fosfolípidos membrana celular, esteroides colesterol, ceras, lípidos complejos</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -6551,7 +6551,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>lípidos parte 3, funciones lípidos, energía, aislamiento, protección, hormonas esteroideas</t>
+          <t>lípidos parte 3, funciones lípidos, energía, aislamiento, protección, hormonas esteroideas, funciones lípidos, reserva energética, aislamiento térmico, protección órganos, hormonas esteroideas</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -6596,7 +6596,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>aminoácidos, péptidos, proteínas, enlace peptídico, estructura primaria, secundaria, terciaria, cuaternaria, desnaturalización</t>
+          <t>aminoácidos, péptidos, proteínas, enlace peptídico, estructura primaria, secundaria, terciaria, cuaternaria, desnaturalización, aminoácidos péptidos proteínas, enlace peptídico, estructura primaria secundaria terciaria cuaternaria, desnaturalización, funciones proteínas</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -6686,7 +6686,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>enzimas, catalizador biológico, sustrato, sitio activo, cofactor, coenzima, inhibición, cinética enzimática</t>
+          <t>enzimas, catalizador biológico, sustrato, sitio activo, cofactor, coenzima, inhibición, cinética enzimática, enzimas catalizadores biológicos, acelerar reacciones químicas, sustrato sitio activo, cofactores coenzimas, cinética enzimática</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>vitaminas, hidrosolubles, liposolubles, vitamina A, B, C, D, E, K, deficiencia, función</t>
+          <t>vitaminas, hidrosolubles, liposolubles, vitamina A, B, C, D, E, K, deficiencia, función, vitaminas biomoléculas esenciales, hidrosolubles liposolubles, clasificación, importancia procesos metabólicos, deficiencias</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -6817,7 +6817,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>membrana celular, bicapa lipídica, modelo mosaico fluido, fosfolípidos, proteínas membrana, permeabilidad selectiva</t>
+          <t>membrana celular, bicapa lipídica, modelo mosaico fluido, fosfolípidos, proteínas membrana, permeabilidad selectiva, membranas biológicas estructura, composición fosfolípidos proteínas carbohidratos, bicapa lipídica, modelo mosaico fluido</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>transporte celular, difusión, ósmosis, transporte activo, pasivo, endocitosis, exocitosis, bomba sodio potasio</t>
+          <t>transporte celular, difusión, ósmosis, transporte activo, pasivo, endocitosis, exocitosis, bomba sodio potasio, modelo mosaico fluido, permeabilidad selectiva, transporte activo pasivo, difusión ósmosis, endocitosis exocitosis</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -6948,7 +6948,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>sistema endomembranas, retículo endoplásmico, aparato Golgi, lisosomas, vesículas, RE liso, RE rugoso</t>
+          <t>sistema endomembranas, retículo endoplásmico, aparato Golgi, lisosomas, vesículas, RE liso, RE rugoso, sistema endomembranas, retículo endoplásmico liso rugoso, aparato Golgi, lisosomas, vesículas, procesamiento proteínas</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -6993,7 +6993,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>citoesqueleto, microtúbulos, microfilamentos, filamentos intermedios, movimiento celular, forma célula</t>
+          <t>citoesqueleto, microtúbulos, microfilamentos, filamentos intermedios, movimiento celular, forma célula, citoesqueleto, microtúbulos microfilamentos filamentos intermedios, forma celular, movimiento, división celular</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -7079,7 +7079,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>mitocondrias, respiración celular, ATP, glucólisis, ciclo Krebs, cadena transporte electrones, fosforilación oxidativa</t>
+          <t>mitocondrias, respiración celular, ATP, glucólisis, ciclo Krebs, cadena transporte electrones, fosforilación oxidativa, mitocondrias respiración celular, ATP producción energía, glucólisis ciclo Krebs, cadena transporte electrones, fosforilación oxidativa</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -7165,7 +7165,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>fotosíntesis, cloroplasto, clorofila, fase luminosa, fase oscura, ciclo Calvin, CO2, O2, glucosa, tilacoides, estroma</t>
+          <t>fotosíntesis, cloroplasto, clorofila, fase luminosa, fase oscura, ciclo Calvin, CO2, O2, glucosa, tilacoides, estroma, fotosíntesis cloroplasto clorofila, fase luminosa oscura, ciclo Calvin, CO2 O2 glucosa, tilacoides estroma, energía solar</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -7251,7 +7251,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>microscopio, microscopía óptica, electrónica, resolución, aumento, preparación muestras, tinción, tipos microscopio</t>
+          <t>microscopio, microscopía óptica, electrónica, resolución, aumento, preparación muestras, tinción, tipos microscopio, microscopio óptico electrónico, resolución aumento, preparación muestras tinción, tipos microscopio, observación células</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -7337,7 +7337,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>mitosis, meiosis, ciclo celular, profase, metafase, anafase, telofase, cromosomas, diploide, haploide, crossing over, gametos</t>
+          <t>mitosis, meiosis, ciclo celular, profase, metafase, anafase, telofase, cromosomas, diploide, haploide, crossing over, gametos, mitosis meiosis ciclo celular, profase metafase anafase telofase, cromosomas diploide haploide, crossing over gametos, división celular</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>tejidos, epitelial, conectivo, muscular, nervioso, histología, clasificación tejidos, funciones</t>
+          <t>tejidos, epitelial, conectivo, muscular, nervioso, histología, clasificación tejidos, funciones, tejidos epitelial conectivo muscular nervioso, histología, clasificación funciones, tipos celulares especializados</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>genética, Mendel, leyes herencia, dominante, recesivo, genotipo, fenotipo, alelos, homocigoto, heterocigoto, Punnett, herencia ligada sexo</t>
+          <t>genética, Mendel, leyes herencia, dominante, recesivo, genotipo, fenotipo, alelos, homocigoto, heterocigoto, Punnett, herencia ligada sexo, genética Mendel leyes herencia, dominante recesivo, genotipo fenotipo, alelos homocigoto heterocigoto, cuadro Punnett, herencia ligada sexo</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Agregar curso Física UCV al chatbot
57 registros (8 lecciones, 49 temas). Cubre magnitudes, vectores, cinemática (MRU, MRUV, caída libre), dinámica (Newton), trabajo-potencia-energía, hidrostática, hidrodinámica y óptica.
Total: 3 cursos, 194 registros.
</commit_message>
<xml_diff>
--- a/quimica_ucv_base_datos.xlsx
+++ b/quimica_ucv_base_datos.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Base de Datos Química UCV" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Base de Datos Biología UCV" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Base de Datos Física UCV" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,8 +52,13 @@
       <color rgb="001B5E20"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001565C0"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +89,18 @@
         <bgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001565C0"/>
+        <bgColor rgb="001565C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BBDEFB"/>
+        <bgColor rgb="00BBDEFB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -102,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -121,6 +139,12 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7526,4 +7550,2609 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Tema/Subtema</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Nombre Completo</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Palabras Clave</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>Descripción para IA</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Magnitudes</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr"/>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Magnitudes</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/magnitudes/</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>magnitudes, unidades, medición, sistema internacional, conversiones</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>Lección sobre magnitudes físicas y unidades de medida</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Magnitudes</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Teoría de Magnitudes</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Magnitudes &gt; Teoría de Magnitudes</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/magnitudes/topics/teoria-de-magnitudes/</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>magnitudes, escalares, vectoriales, unidades, SI, medición, dimensiones, conversión unidades</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Teoría de magnitudes: escalares, vectoriales, unidades del SI, conversiones</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Magnitudes</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Magnitudes Vectoriales</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Magnitudes &gt; Magnitudes Vectoriales</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/magnitudes/topics/magnitudes-vectoriales/</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>magnitudes vectoriales, dirección, sentido, módulo, representación gráfica, vectores introducción</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Magnitudes vectoriales: dirección, sentido, módulo y representación gráfica</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>vectores, suma vectores, resultante, descomposición, ángulo, física vectorial</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Lección completa sobre vectores: operaciones, descomposición, resultantes</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Introducción a Vectores</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Introducción a Vectores</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/introduccion-a-vectores-3/</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>vectores, qué son, representación gráfica, módulo dirección sentido, física fundamental</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Qué son los vectores, representación gráfica, módulo, dirección y sentido</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Cómo se Descompone un Vector</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Cómo se Descompone un Vector</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/como-se-descompone-un-vector/</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>descomposición vectorial, componentes x y, seno coseno, eje cartesiano, proyecciones</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Descomposición de un vector en componentes x e y usando seno y coseno</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Formas de Representar un Vector Parte 1</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Formas de Representar un Vector Parte 1</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/formas-de-representar-un-vector-parte-1/</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>representar vector, forma polar, forma cartesiana, módulo ángulo, componentes</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Formas de representar un vector: polar y cartesiana, módulo y ángulo</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Formas de Representar un Vector Parte 2</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Formas de Representar un Vector Parte 2</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/formas-de-representar-un-vector-parte-2/</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>representar vector parte 2, conversión polar cartesiana, vectores unitarios, notación</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Conversión entre representaciones polares y cartesianas de vectores</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Qué es una Resultante</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Qué es una Resultante</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/que-es-una-resultante/</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>resultante, suma vectores, vector resultante, efecto neto, fuerzas</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Qué es la resultante de vectores: suma vectorial y efecto neto</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Resultante por Descomposición Cartesiana</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Resultante por Descomposición Cartesiana</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/resultante-por-descomposicion-cartesiana/</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>resultante descomposición cartesiana, sumar componentes x y, método analítico, cálculo resultante</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Calcular la resultante descomponiendo vectores en componentes x e y</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Resultante y Diferencia de Vectores</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Resultante y Diferencia de Vectores</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/resultante-y-diferencia-de-vectores/</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>resultante diferencia vectores, resta vectorial, vector opuesto, suma resta</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Resultante y diferencia de vectores: resta vectorial y vector opuesto</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Ángulo Entre Dos Vectores</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Ángulo Entre Dos Vectores</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/angulo-entre-dos-vectores/</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>ángulo entre vectores, producto escalar, coseno ángulo, relación vectores</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Cálculo del ángulo entre dos vectores usando producto escalar</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Resultante Máxima y Mínima</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Resultante Máxima y Mínima</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/resultante-maxima-y-minima/</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>resultante máxima mínima, vectores mismo sentido opuesto, suma resta módulos</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Resultante máxima (mismo sentido) y mínima (sentido opuesto) de vectores</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Vectores</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Ejercicio Con Baricentro</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Vectores &gt; Ejercicio Con Baricentro</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/vectores/topics/ejercicio-con-baricentro/</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>baricentro, centro gravedad, centro masa, triángulo, coordenadas medias</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Ejercicio de baricentro: centro de gravedad y coordenadas medias</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr"/>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>cinemática, movimiento, MRU, MRUV, caída libre, tiro vertical, gráficos</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Lección completa sobre cinemática: MRU, MRUV, caída libre, gráficos</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>MRU Conceptos Claves</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; MRU Conceptos Claves</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/movimiento-rectilineo-uniforme-concepto-claves/</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>MRU, movimiento rectilíneo uniforme, velocidad constante, línea recta, posición tiempo distancia</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>MRU: cuerpo se desplaza en línea recta con velocidad constante</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Sistema de Referencia y Velocidad Media</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; Sistema de Referencia y Velocidad Media</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/sistema-de-referencia-y-velocidad-media/</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>sistema referencia, velocidad media, desplazamiento tiempo, punto referencia, observador</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Sistema de referencia y velocidad media: desplazamiento sobre tiempo</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Velocidad Media vs Rapidez Media</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; Velocidad Media vs Rapidez Media</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/velocidad-media-vs-rapidez-media/</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>velocidad media, rapidez media, diferencia, escalar vectorial, distancia desplazamiento</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Diferencia entre velocidad media (vectorial) y rapidez media (escalar)</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Gráficos Posición vs Tiempo MRU</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; Gráficos Posición vs Tiempo MRU</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/graficos-de-posicion-en-funcion-al-tiempo-del-mru/</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>gráfico posición tiempo MRU, pendiente velocidad, recta, interpretar gráficos cinemática</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Interpretar gráficos posición vs tiempo del MRU: pendiente = velocidad</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Gráfico Velocidad vs Tiempo MRU</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; Gráfico Velocidad vs Tiempo MRU</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/grafico-de-velocidad-en-funcion-al-tiempo-del-mru/</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>gráfico velocidad tiempo MRU, recta horizontal, área desplazamiento, constante</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Gráfico velocidad vs tiempo del MRU: recta horizontal, área = desplazamiento</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>MRUV Velocidad en Función del Tiempo</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; MRUV Velocidad en Función del Tiempo</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/m-r-u-v-velocidad-en-funcion-del-tiempo/</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>MRUV, velocidad función tiempo, aceleración constante, acelerar desacelerar, v=v0+at</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>MRUV: velocidad en función del tiempo, aceleración constante, v=v0+at</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>MRUV Posición en Función del Tiempo</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; MRUV Posición en Función del Tiempo</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/m-r-u-v-posicion-en-funcion-al-tiempo/</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>MRUV posición tiempo, ecuación horaria, parábola, x=x0+v0t+½at², desplazamiento</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>MRUV: posición en función del tiempo, ecuación horaria x=x0+v0t+½at²</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Ecuación de Torricelli</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; Ecuación de Torricelli</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/ecuacion-de-torricelli/</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Torricelli, ecuación sin tiempo, v²=v0²+2aΔx, MRUV, velocidad posición aceleración</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Ecuación de Torricelli: v²=v0²+2aΔx, relaciona velocidad posición y aceleración sin tiempo</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Gráfico Posición vs Tiempo MRUV</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; Gráfico Posición vs Tiempo MRUV</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/grafico-de-posicion-en-funcion-al-tiempo-del-mruv/</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>gráfico posición tiempo MRUV, parábola, concavidad, aceleración, interpretar</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Gráfico posición vs tiempo del MRUV: parábola, concavidad indica aceleración</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Gráfico Velocidad vs Tiempo MRUV</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; Gráfico Velocidad vs Tiempo MRUV</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/grafico-de-velocidad-en-funcion-al-tiempo-del-mruv/</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>gráfico velocidad tiempo MRUV, recta inclinada, pendiente aceleración, área desplazamiento</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Gráfico velocidad vs tiempo del MRUV: recta inclinada, pendiente = aceleración</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Caída Libre y Tiro Vertical</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; Caída Libre y Tiro Vertical</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/caida-libre-y-tiro-vertical/</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>caída libre, tiro vertical, gravedad 9.8 m/s², aceleración gravitatoria, altura tiempo velocidad</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Caída libre y tiro vertical: gravedad 9.8 m/s², ecuaciones de movimiento vertical</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Interpretación Interactiva de Gráficos</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Cinemática &gt; Interpretación Interactiva de Gráficos</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/cinematica/topics/interpretacion-interactiva-de-graficos/</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>gráficos interactivos, simulación, cinemática, interpretar movimiento, posición velocidad</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Interpretación interactiva de gráficos de cinemática con simulaciones</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr"/>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>dinámica, fuerzas, leyes Newton, DCL, equilibrio, fuerzas oblicuas</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>Lección sobre dinámica: leyes de Newton, fuerzas, equilibrio, DCL</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica Concepto</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica &gt; Dinámica Concepto</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/topics/dinamica-concepto/</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>dinámica concepto, fuerza, masa, aceleración, causa movimiento, interacción</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Concepto de dinámica: estudio de las fuerzas como causa del movimiento</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio de un Cuerpo</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica &gt; Equilibrio de un Cuerpo</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/topics/equilibrio-de-un-cuerpo/</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>equilibrio, fuerza neta cero, estático dinámico, condiciones equilibrio, reposo</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Equilibrio de un cuerpo: fuerza neta igual a cero, equilibrio estático y dinámico</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Primera Ley de Newton</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica &gt; Primera Ley de Newton</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/topics/primera-ley-de-newton/</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>primera ley Newton, inercia, cuerpo reposo movimiento, fuerza neta cero, tendencia mantener estado</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Primera ley de Newton (inercia): un cuerpo mantiene su estado si la fuerza neta es cero</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Segunda Ley de Newton</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica &gt; Segunda Ley de Newton</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/topics/segunda-ley-de-newton/</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>segunda ley Newton, F=ma, fuerza masa aceleración, relación directa inversa</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Segunda ley de Newton: F=ma, la fuerza es proporcional a masa × aceleración</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Tercera Ley de Newton</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica &gt; Tercera Ley de Newton</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/topics/tercera-ley-de-newton/</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>tercera ley Newton, acción reacción, pares fuerzas, igual magnitud sentido opuesto</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Tercera ley de Newton: acción y reacción, fuerzas iguales en sentido opuesto</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Repaso + DCL</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica &gt; Repaso + DCL</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/topics/repaso-dcl/</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>DCL, diagrama cuerpo libre, fuerzas sobre cuerpo, normal peso fricción tensión, repaso</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Diagrama de cuerpo libre (DCL): identificar todas las fuerzas sobre un cuerpo</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Fuerzas Oblicuas</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica &gt; Fuerzas Oblicuas</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/topics/fuerzas-oblicuas/</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>fuerzas oblicuas, fuerza inclinada, componentes, plano inclinado, descomposición fuerza ángulo</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Fuerzas oblicuas: descomposición de fuerzas inclinadas en componentes</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Práctica de DCL</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica &gt; Práctica de DCL</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/topics/practica-dcl/</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>práctica DCL, ejercicios diagrama cuerpo libre, identificar fuerzas, resolver problemas</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Práctica de diagramas de cuerpo libre: ejercicios para identificar fuerzas</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica Retroalimentación Conceptual</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Dinámica &gt; Dinámica Retroalimentación Conceptual</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/dinamica/topics/dinamica-retroalimentacion-conceptual/</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>retroalimentación dinámica, repaso conceptos, leyes Newton resumen, fuerzas aplicaciones</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Retroalimentación conceptual de dinámica: repaso de leyes de Newton y aplicaciones</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Trabajo-Potencia-Energía</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr"/>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>Trabajo-Potencia-Energía</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/trabajo-potencia-energia/</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>trabajo, potencia, energía, cinética, potencial, mecánica, conservación</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>Lección sobre trabajo, potencia y energía en física</t>
+        </is>
+      </c>
+      <c r="I39" s="9" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Trabajo-Potencia-Energía</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Trabajo y Potencia</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Trabajo-Potencia-Energía &gt; Trabajo y Potencia</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/trabajo-potencia-energia/topics/trabajo-y-potencia-2/</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>trabajo físico, potencia, fuerza desplazamiento, joule, watt, transferir energía, W=Fd cosθ</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Trabajo físico (W=Fd cosθ) y potencia (P=W/t): transferencia de energía</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Trabajo-Potencia-Energía</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Trabajo-Potencia-Energía &gt; Energía</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/trabajo-potencia-energia/topics/energia-2/</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>energía, cinética, potencial gravitatoria, mecánica, conservación energía, transformación, ½mv²</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Energía cinética (½mv²), potencial gravitatoria (mgh), mecánica y conservación</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr"/>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>hidrostática, presión, fluidos, densidad, empuje, Arquímedes, Pascal</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>Lección sobre hidrostática: presión, densidad, empuje en fluidos</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Densidad de un Líquido</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Densidad de un Líquido</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/densidad-de-un-liquido/</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>densidad, masa volumen, ρ=m/V, comparar sustancias, kg/m³, g/cm³</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Densidad: ρ=m/V, comparar cuánta materia hay en el mismo volumen</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Presión de una Fuerza</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Presión de una Fuerza</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/presion-de-una-fuerza/</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>presión, fuerza área, P=F/A, pascal, superficie, distribuir fuerza</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Presión: P=F/A, fuerza distribuida sobre una superficie</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Presión de un Líquido</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Presión de un Líquido</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/presion-de-un-liquido/</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>presión hidrostática, P=ρgh, profundidad, densidad gravedad, columna líquido</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Presión hidrostática: P=ρgh, depende de densidad, gravedad y profundidad</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Presión Atmosférica</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Presión Atmosférica</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/presion-atmosferica/</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>presión atmosférica, 1 atm, 101325 Pa, Torricelli, columna mercurio, altitud</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Presión atmosférica: 1 atm = 101325 Pa, experimento de Torricelli</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Presión Total</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Presión Total</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/presion-total/</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>presión total, presión absoluta, atmosférica + hidrostática, manométrica, Ptotal</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Presión total = atmosférica + hidrostática, presión absoluta y manométrica</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Teorema de Stevin</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Teorema de Stevin</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/teorema-de-stevin/</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Stevin, diferencia presiones, puntos mismo líquido, profundidad, ΔP=ρgΔh</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Teorema de Stevin: la diferencia de presiones depende de la diferencia de profundidad</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Teorema de Pascal</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Teorema de Pascal</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/teorema-de-pascal/</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Pascal, presión transmite igual, fluido cerrado, prensa hidráulica, multiplicar fuerza</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Teorema de Pascal: la presión se transmite igual en todas las direcciones en un fluido cerrado</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Vasos Comunicantes</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Vasos Comunicantes</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/vasos-comunicantes/</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>vasos comunicantes, mismo nivel, mismo líquido, presión equilibrio, conectados</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Vasos comunicantes: líquidos al mismo nivel cuando están conectados</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Empuje de un Líquido</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Empuje de un Líquido</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/empuje-de-un-liquido/</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>empuje, Arquímedes, fuerza ascendente, peso líquido desplazado, flotar hundir, E=ρVg</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Empuje (Arquímedes): fuerza ascendente = peso del líquido desplazado, E=ρVg</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Aceleración dentro de un Líquido</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Hidrostática &gt; Aceleración dentro de un Líquido</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrostatica/topics/aceleracion-dentro-de-un-liquido/</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>aceleración líquido, objeto sumergido, gravedad empuje peso, velocidad fluido</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Aceleración de un objeto dentro de un líquido: efecto de gravedad y empuje</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Hidrodinámica</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr"/>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>Hidrodinámica</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrodinamica/</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>hidrodinámica, fluidos movimiento, Bernoulli, caudal, continuidad</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>Lección sobre hidrodinámica: fluidos en movimiento</t>
+        </is>
+      </c>
+      <c r="I53" s="9" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Hidrodinámica</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Hidrodinámica Conceptos Claves</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Hidrodinámica &gt; Hidrodinámica Conceptos Claves</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/hidrodinamica/topics/hidrodinamica-conceptos-claves/</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>hidrodinámica, caudal, ecuación continuidad, Bernoulli, flujo laminar turbulento, tubo corriente</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Conceptos de hidrodinámica: caudal, ecuación de continuidad, Bernoulli</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>Lección</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>Óptica</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="inlineStr"/>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>Óptica</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/optica/</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>óptica, espejos, reflexión, luz, imagen, esféricos, planos</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>Lección sobre óptica: espejos planos y esféricos</t>
+        </is>
+      </c>
+      <c r="I55" s="9" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Óptica</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Espejos Planos Conceptos</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Óptica &gt; Espejos Planos Conceptos</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/optica/topics/espejos-planos-conceptos/</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>espejos planos, reflexión, imagen virtual, simétrica, leyes reflexión, normal</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Espejos planos: reflexión, imagen virtual y simétrica, leyes de reflexión</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Óptica</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Espejos Esféricos Conceptos</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Óptica &gt; Espejos Esféricos Conceptos</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/optica/topics/espejos-esfericos-conceptos/</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>espejos esféricos, cóncavo convexo, foco, centro curvatura, radio, imagen real virtual</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Espejos esféricos: cóncavos y convexos, foco, centro de curvatura, tipos de imagen</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Óptica</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Rayos Notables Espejos Esféricos</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Óptica &gt; Rayos Notables Espejos Esféricos</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>https://idappi.com/courses/fisicaidappi/lessons/optica/topics/rayos-notables-espejos-esfericos/</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>rayos notables, espejos esféricos, paralelo foco, centro curvatura, construcción imagen, trazado</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Rayos notables en espejos esféricos: trazado de rayos para construir imágenes</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Física UCV</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>